<commit_message>
Investigación plantillas cerámicas: competencia por país y tracker actualizado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tBz94YMaY7YngtLZRe8ni
</commit_message>
<xml_diff>
--- a/research/productos-investigados.xlsx
+++ b/research/productos-investigados.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:W42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3840,6 +3840,1205 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>The Clay Blueprints</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pack de plantillas imprimibles (EN)</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>90</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>GANADOR FUERTE</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>34</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>EN · US/GB/DE/AU + Europa del Este</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>10</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>sí (en inglés)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>~US$42 (Dhs 154, según Excel unificado)</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>EE. UU./Reino Unido; no recomendado para entrar ahora (mercado inglés con ~10 clones)</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>→ estable (34 ads, igual que el Excel unificado del 7-oct)</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>1343302345522178</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1692912678840741</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PrintClay Studio</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Plantillas pre-dimensionadas (EN/FR/NL/DA)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>90</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>GANADOR FUERTE</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>33</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>EN, FR, NL, DA · EE. UU. + Europa</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>10</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>sí (en inglés)</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Francia y Países Bajos: lo está traduciendo y testeando</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>1097177920156365</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1140551188635978</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>La Biblia de las Plantillas Cerámicas — Ceramicaemprendedor</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Biblia de plantillas (ES/EN/DE)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>86</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>GANADOR FUERTE</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="J34" t="n">
+        <v>75</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ES, EN, DE · LATAM + España + EE. UU.</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>5</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>España y México (es el líder hispano; página con 1005 anuncios activos, multi-producto)</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>860004577196412</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1414645386715189</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kit de Plantillas Cerámicas — HI MERY</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Kit de plantillas + bonos</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>71</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J35" t="n">
+        <v>26</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ES · MX, ES, CL, CO, PE, UY, US (no pauta en AR)</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>5</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>No verificado (anuncio '50% OFF + 7 bonos')</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Chile y España (mismo alcance que el producto del usuario, sin AR)</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>106784294503235</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1631515018383419</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ClayLab DIY / ClayCraft DIY (mismo operador)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>30+ plantillas imprimibles (EN/DE)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>68</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J36" t="n">
+        <v>21</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>EN, DE · Europa</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>sí (en inglés)</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Alemania</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>978035102055668</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1397995229163204</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pottery Blueprint</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Plantillas de papel para cerámica (EN)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>66</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>16</v>
+      </c>
+      <c r="J37" t="n">
+        <v>5</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>EN · Europa (EUR)</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>10</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>sí (en inglés)</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Reino Unido/Irlanda</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>1339142019281477</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1134164862604217</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Clay Maker Lab</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Plantillas 'no wheel' (EN)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>58</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="J38" t="n">
+        <v>8</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>EN · Europa (EUR)</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>10</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>sí (en inglés)</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Europa del norte</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>1327089017144597</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1060421846815507</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sistema Arcilla en Casa</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Método arcilla sin horno ni torno (ES)</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>56</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>6</v>
+      </c>
+      <c r="J39" t="n">
+        <v>5</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ES · LATAM + España + EE. UU.</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>5</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>1353864484479328</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1808767807134186</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Barro Club</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>+40 plantillas PDF para clases (ES)</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>42</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ES · Argentina</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>5</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Argentina (profes de talleres)</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>1050393238168035</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=2880014209043327</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Armá tu propia línea de cerámica — Ebooks del Futuro</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Ebook/kit emprendimiento cerámica (ES)</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>41</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" t="n">
+        <v>9</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ES · Argentina</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>5</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>725759253957744</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=938026992362764</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plantillas para cerámica — Pulso cerámica</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Cerámica / plantillas</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Plantillas (ES, cobra en ARS)</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>41</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Chequeo cerámica 10-oct</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" t="n">
+        <v>8</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ES · Argentina</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>5</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Bajo (sin claims de salud/ingresos detectados en títulos)</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Mujeres 30-60 que hacen cerámica de placa (slab) sin torno</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad: cortar piezas a medida sin deformar ni desperdiciar arcilla</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>269424112913360</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1760679795236946</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Marcar Ebooks del Futuro como producto propio del usuario
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tBz94YMaY7YngtLZRe8ni
</commit_message>
<xml_diff>
--- a/research/productos-investigados.xlsx
+++ b/research/productos-investigados.xlsx
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Armá tu propia línea de cerámica — Ebooks del Futuro</t>
+          <t>Armá tu propia línea de cerámica — Ebooks del Futuro (PRODUCTO PROPIO)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4842,17 +4842,14 @@
           <t>Ebook/kit emprendimiento cerámica (ES)</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v>41</v>
-      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>POTENCIAL</t>
+          <t>PROPIO (no es competencia)</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -4911,12 +4908,12 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Test actual en AR; próximos: España y Chile</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Primer chequeo</t>
+          <t>Lanzado 9-oct: 2 ventas con US$5</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">

</xml_diff>

<commit_message>
Cacería 13-oct: 20 infoproductos en ascenso, top 3 ES y top 3 otros idiomas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tBz94YMaY7YngtLZRe8ni
</commit_message>
<xml_diff>
--- a/research/productos-investigados.xlsx
+++ b/research/productos-investigados.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W42"/>
+  <dimension ref="A1:W62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5036,6 +5036,2186 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Aprende a leer jugando 🦉 — Neurokids1 (red de 6 páginas)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Infantil / lectura</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pack lúdico de lectoescritura</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>61</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J43" t="n">
+        <v>38</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>PL, IT, CZ, RO, GR, FR, ES (red ~92 ads)</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Madres 28-45 con hijos de 4-7 años; abuelas 50-65 que regalan</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad (hijo que no arranca a leer)</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>España, Chile, Uruguay, EE. UU. hispano</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>1125298484000687</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1630068381827850</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>160 recetas para tu Ninja Crispi — Cocina con Lola</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Cocina / electrodoméstico</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Recetario PDF</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>56</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J44" t="n">
+        <v>33</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ES, DE, EN, FR</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Medio: marca registrada 'Ninja' en anuncios</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Mujeres 35-60 que compraron o recibieron la Ninja Crispi</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Problema concreto: sacarle partido al aparato</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>España, EE. UU. hispano, México, Chile</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>899211696601502</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1615453983318240</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>8 perros hiperrealistas al crochet — Crochet Pro</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Crochet / amigurumi</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Patrones PDF</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>46</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J45" t="n">
+        <v>26</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Mujeres 35-65 tejedoras con nivel medio, amantes de perros</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad / regalo personalizado</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>España, México, Chile, Argentina (en español no hay oferta)</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>1177673052104302</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1668371231538712</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>150 Boutique Gift Baskets — Berenice Garcia</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Negocio desde casa / eventos</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Libro de ideas (serie)</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>55</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J46" t="n">
+        <v>79</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>EN (US)</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Bajo: evitar promesas de ingresos</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Mujeres 35-60 que quieren un ingreso extra con regalos/eventos</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Ingresos extra (temporada de regalos)</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>EE. UU., Canadá, Australia, Reino Unido; luego español</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>1087168021148527</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1443117621217189</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>150 fichas de anatomía para colorear — Printora</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Estudio / salud</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Fichas imprimibles</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>66</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="J47" t="n">
+        <v>34</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>FR, IT, DE, EN</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>2</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Estudiantes de enfermería/medicina/veterinaria 18-35</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Aprender (memorizar anatomía)</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Alemania, Países Bajos, Polonia, nórdicos (español ya saturado)</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>1232916199911605</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1124664126802508</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>500 actividades para adultos mayores — Digital Corner (+Bookbay SK)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Cuidado de mayores</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Pack imprimible</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>59</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" t="n">
+        <v>32</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>HU, SK</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Hijas 40-65 que cuidan a padres mayores; animadoras de residencias</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Problema concreto: entretener/estimular a un mayor</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Alemania, Italia, España, Polonia, nórdicos</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>1358074294058687</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1829682791389006</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Ruhe im Kopf (sobrepensamiento) — Ruhe im Kopf</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bienestar mental</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Guía (formato ?)</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>61</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="J49" t="n">
+        <v>38</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
+        <v>4</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Medio: claims de salud mental</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Mujeres 35-55 con estrés y rumiación</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Problema concreto: calmar la mente</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Alemania, Austria, Suiza</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>1277187975474703</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1098550906254228</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Explicado en dibujos (ebooks de estudio) — Étudefacile</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Estudio / formación</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Ebooks ilustrados</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>50</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="J50" t="n">
+        <v>40</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>FR (+IT/ES vía Studio Facile)</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Estudiantes 18-35 de oficios y salud</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Aprender más rápido</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Alemania, Países Bajos, Polonia</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>1299578486577349</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1743486216949015</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>3 libros, 1 precio (niños: acoso y normas) — Digital Club Edu</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Crianza</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pack de libros infantiles</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>61</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="J51" t="n">
+        <v>54</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>CS, RO, EL, PT(€)</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Madres 30-45 de niños 5-10</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Problema concreto: acoso escolar</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Polonia, Hungría, Alemania, España</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>1361301167057013</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1419550166952042</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000 porqués (preguntas y respuestas) — Ezer Miért / Bin Neden</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Infantil / curiosidad</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Libro infantil</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>49</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J52" t="n">
+        <v>52</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>HU, TR</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Padres 30-45 de niños 5-10</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Aprender</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Polonia, Rumanía, España</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>1340954699103216</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1427285042193505</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>500.000+ diseños de sublimación — Tu Ebook Favorito</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sublimación / POD</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Megapack de diseños</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>51</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J53" t="n">
+        <v>160</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>PL, RO, CS, PT</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Medio: derechos de diseños de terceros</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Emprendedoras 25-50 con sublimadora</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Ingresos extra</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Polonia, Chequia, Rumanía</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>1153819164474182</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1105926468862231</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20 enigmas de detective para imprimir — Agenzia dei Piccoli Detective</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Infantil sin pantallas</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Imprimibles</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>46</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="J54" t="n">
+        <v>15</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>2</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Madres 30-45 de niños 6-12</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Problema concreto: menos pantallas</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Italia, España (solo Mentes Mágicas)</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>1440381472481078</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=3700761470091822</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>150 experimentos de química sin laboratorio — Lauren Phillips</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Infantil / ciencia</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Guía de experimentos</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>51</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J55" t="n">
+        <v>33</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Madres homeschool 30-45</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Aprender</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>EE. UU., Reino Unido, Australia (español ya competido)</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>1301771929686425</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=977580018744582</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>200 patrones de corsé / 50 velas comestibles — Practical Guides</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Costura / velas</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Patrones + recetario</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>63</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="J56" t="n">
+        <v>67</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Mujeres 30-55 costureras/hobby</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Aprender una habilidad</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>EE. UU., Reino Unido, Alemania</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>1280447521827796</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=2271474530341702</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>300 problemas de ajedrez — The Knight's Notebook</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ajedrez</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cuadernos imprimibles</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>54</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J57" t="n">
+        <v>22</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>NO, IT, FR, EN</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Padres y abuelos 35-70 de niños ajedrecistas</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Aprender</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Noruega, Dinamarca, Alemania, Países Bajos</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>1353979041129771</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1457546913012397</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1.200 planos de acero para soldar / juguetes de madera — Mario Rossi</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bricolaje / soldadura</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pack de planos</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>51</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J58" t="n">
+        <v>44</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>NL, IT</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Hombres 35-65 con taller en casa</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Ingresos extra / hobby</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Países Bajos, Alemania, nórdicos</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>1393906473803532</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1802993204071163</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Cajas de chocolatería hechas en tu cocina — Gemas Digitales</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Repostería / emprender</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Curso/guía</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>51</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="J59" t="n">
+        <v>41</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Bajo: evitar promesas de ingresos</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Mujeres 30-55 que quieren vender bombones en Navidad</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Ingresos extra</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>España, México, Chile</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>1129458703589779</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1130908282644296</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Guía de poses 1.200 fichas — Arte Digital</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Fichas de poses</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>66</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="J60" t="n">
+        <v>95</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>FR, IT, EN, ES, JP</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>1</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Fotógrafas aficionadas 25-45</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Aprender</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Alemania, Países Bajos, Polonia</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>276718215524267</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1117079470773438</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Diario imprimible para fe complicada — Still Waters Journals</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Fe / journaling</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Diario imprimible</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>46</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="J61" t="n">
+        <v>22</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Mujeres cristianas 30-60 heridas por la iglesia</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Problema concreto: reconciliar la fe</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>EE. UU., Canadá</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>108018278680669</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1423484263182533</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>210+ patrones de marroquinería — Leathercraft Lab</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Cuero</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Patrones PDF</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>51</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Cacería en ascenso 13-oct</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J62" t="n">
+        <v>20</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com no accesible)</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Hombres y mujeres 30-60 con hobby del cuero</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Aprender / ingresos extra</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>EE. UU., Alemania, nórdicos</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Primer chequeo</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>927974923725307</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=1841735747171829</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel unificado 19-oct: re-chequeo en Ad Library y top 3 para caja rápida
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011tBz94YMaY7YngtLZRe8ni
</commit_message>
<xml_diff>
--- a/research/productos-investigados.xlsx
+++ b/research/productos-investigados.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W62"/>
+  <dimension ref="A1:W80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7216,6 +7216,1462 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Cajas de chocolatería hechas en tu cocina — Gemas Digitales</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>71</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>≥17,5</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>53</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ES · USD</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2-3 directos (Tentaciones Dulces, Sofia Fernández, Aprende Online en Casa)</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>↑ 41 → 53 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>1129458703589779</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>50 Edible Candle Recipes / 200+ Corset Patterns — Practical Guides</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>66</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>≥1,8 (muestra)</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>157</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>EN · USD + COP</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Velas comestibles: ninguno visto (velas genéricas: saturado)</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>↑ 67 → 157 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>1280447521827796</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>150 Boutique Gift Baskets — Berenice Garcia</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="n">
+        <v>60</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>≥10,9</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>82</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>EN · USD</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>1 directo: Canastas que Garpan (6 ads); Emprende con Arte y Club creativo digital, adyacentes</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>↑ 79 → 82 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>1087168021148527</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>La Biblia de las Plantillas Cerámicas — Ceramicaemprendedor</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="n">
+        <v>90</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>GANADOR FUERTE</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>≥10,5</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>583</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ES, IT, FR, NL, CZ, KR, ZH, GR, DK · USD</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Líder del nicho (56 activos en España)</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>↑ 75 → 583 (2026-10-10)</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>860004577196412</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Printable WITH Lisa (workbooks terapia + fe)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>85</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>GANADOR FUERTE</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>≥6,2 (muestra)</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>110</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>EN · USD</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>No buscado</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>↑ 79 → 110 (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>106064502120864</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>3 libros, 1 precio (niños) + tarot — Digital Club Edu</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>71</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>≥5,1 (muestra)</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>161</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>HR, SK, CZ, HU, GR, PT, RO, IT, FR, ES · USD/EUR/HUF</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>No buscado</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>↑ 54 → 161 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>1361301167057013</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>160 recetas para tu Ninja Crispi — Cocina con Lola</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>66</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>12,9</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>47</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ES (+ versión MX), FR · USD</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Recetas freidora: Estante ebooks 6, Recetas con Rosa 4, Hogar y Bienestar 3, otros</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>↑ 33 → 47 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>899211696601502</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Guía de poses 1.200 fichas — Arte Digital</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>68</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>≥5,0 (muestra)</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>104</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ES, FR, EN, JA · USD</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Ya vende su propia versión en español</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>↑ 95 → 104 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>276718215524267</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Ruhe im Kopf (sobrepensamiento)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>66</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>≥12,3</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>56</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>DE · EUR</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>No buscado</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>↑ 38 → 56 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>1277187975474703</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>150 fichas de anatomía para colorear — Printora</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>62</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>GANADOR (saturado en ES)</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>≥0,9 (muestra)</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>453</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>SV, HU, CS, JA, EN, ES · USD</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>~10 vendedores (Printora 14, Vetsemestresse 7, Bela IA 6, Anatomika 5…)</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>↑ 34 → 453 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>1232916199911605</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Universo do Feltro (50 X em Feltro)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="n">
+        <v>65</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>GANADOR (saturado en ES)</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>≥39,8</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>66</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>PT · BRL</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>9+ vendedores (Navidad creativa 15, Aprendia 8, Fieltro en Casa 5…)</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>→ 66 → 66 (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>1438504236004203</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>100 Fichas de Fallas de Aire Acondicionado (HVAC)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="n">
+        <v>60</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>GANADOR</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>44,9</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>26</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ES, IT · USD</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Pocos (Reparación en una Hoja 2, Fuentes Master 1)</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>↓ 38 → 26 (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>1240543665811323 / 1263645906829394</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>210+ patrones de marroquinería — Leathercraft Lab</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>48</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>16,9</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>19</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>EN · EUR</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Se llenó: The Leathercraft Master 11 (hoy), Molderia Studio 7, Maestros del Cuero 5…</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>→ 20 → 19 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>927974923725307</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>100 Attività Sensoriali — Crescere Giocando</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>45</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>9</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>IT · EUR</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Manitoscuriosas.ar 4, Cerebritos 3, NeuroAprendizaje 2</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>↓ 22 → 9 (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>1009883552206401</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Aprende a leer jugando — Neurokids1 / El búho Leo</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>40</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>POTENCIAL</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>10,5</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>15</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>IT, PL · USD (español apagado)</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Ninguno directo</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>↓ 38 → 15 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>1125298484000687 / 1406400125885793</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>8 perros hiperrealistas al crochet — Crochet Pro</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="n">
+        <v>30</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>DESCARTAR</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>11,6</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>14</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>FR · USD</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Casi nadie</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>↓ 26 → 14 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>1177673052104302</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>500 actividades para adultos mayores — Digital Corner</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="n">
+        <v>25</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>DESCARTAR</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>0,9</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>29</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>HU, CS, IT · USD</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>6+ vendedores en español</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>↓ 32 → 29 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>1358074294058687</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Ebooks del Futuro (TU página)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>PROPIO</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Re-chequeo 19-oct</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>≥5,7 (muestra)</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>69</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ES (tú + voseo) · USD</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>No verificada (facebook.com y landings no accesibles)</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>No verificado</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>↑ 9 → 69 (2026-10-10)</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>725759253957744</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>